<commit_message>
Package C: coordinate import semantics (xls/xlsx/csv + field mapping + traceability + CoordinateMeaningConfirmed gating), 14 new tests
87 tests green; synthetic PASS/NG/NG unchanged; pcb_config.xlsx migrated to extended template
</commit_message>
<xml_diff>
--- a/data/pcb_config.xlsx
+++ b/data/pcb_config.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:AC7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,6 +509,71 @@
           <t>RoiExpand</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>PartNumber</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>X_Offset</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Y_Offset</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>TeachX</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>TeachY</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>TeachAngle</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>CoordinateSystem</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>CoordinateMeaningConfirmed</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>BoardID</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>SourceFile</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>SourceSheet</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>SourceRow</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -569,6 +634,47 @@
       <c r="P2" t="n">
         <v>0.2</v>
       </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="U2" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>pcb_absolute_mm</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>BOARD_1</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>合成模板(自建几何,语义已定义)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -629,6 +735,47 @@
       <c r="P3" t="n">
         <v>0.2</v>
       </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>35</v>
+      </c>
+      <c r="U3" t="n">
+        <v>50</v>
+      </c>
+      <c r="V3" t="n">
+        <v>90</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>pcb_absolute_mm</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>BOARD_1</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>合成模板(自建几何,语义已定义)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -689,6 +836,47 @@
       <c r="P4" t="n">
         <v>0.2</v>
       </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="U4" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="V4" t="n">
+        <v>90</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>pcb_absolute_mm</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>BOARD_1</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>合成模板(自建几何,语义已定义)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -749,6 +937,47 @@
       <c r="P5" t="n">
         <v>0.2</v>
       </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>60</v>
+      </c>
+      <c r="U5" t="n">
+        <v>55</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>pcb_absolute_mm</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>BOARD_1</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>合成模板(自建几何,语义已定义)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -809,6 +1038,47 @@
       <c r="P6" t="n">
         <v>0.2</v>
       </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>50</v>
+      </c>
+      <c r="U6" t="n">
+        <v>40</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>pcb_absolute_mm</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>BOARD_1</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>合成模板(自建几何,语义已定义)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -868,6 +1138,47 @@
       </c>
       <c r="P7" t="n">
         <v>0.2</v>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>75</v>
+      </c>
+      <c r="U7" t="n">
+        <v>25</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>pcb_absolute_mm</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>BOARD_1</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>合成模板(自建几何,语义已定义)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>